<commit_message>
Sprint 2: acceso a la cuenta, asistente de perfil, 4+1 en UML y reorganizacion segun el docente
- FS-HU-15, FS-HU-17, FS-HU-18 y FS-HU-19 implementadas; FS-HU-16 (Google) en espera

- Codigo trasladado a FASE 2/Evidencias Proyecto/Evidencias de sistema; capturas en Evidencias de documentacion/Sprint N

- Documentacion: DAS v1.10, DoD v1.5, Guia 2.4, backlog, casos de prueba 19/19, defectos y Sprint Backlog 2 (borrador)
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I18"/>
+  <dimension ref="B1:I23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" style="5" min="1" max="1"/>
@@ -1049,6 +1049,196 @@
       <c r="I18" s="9" t="inlineStr">
         <is>
           <t>Agregada el 15-09-2026 (épica E7 Reservas). Al presionar "Reservar" el usuario escribe un mensaje breve obligatorio para el profesional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-15</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario, necesito recuperar mi contraseña mediante un enlace enviado a mi correo, con la finalidad de volver a acceder a mi cuenta si la olvido.</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Recuperar contraseña</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 21-09-2026 (épica E1) por decisión del Product Owner, a partir del diseño de las pantallas de acceso. El enlace vence a los 60 minutos y sirve una sola vez. 21-09-2026: implementada y probada (CP-011 a CP-013); falta configurar la cuenta de correo SMTP para el envío real y completar la DoD (revisión de código y PR).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-16</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario o profesional, necesito registrarme e iniciar sesión con mi cuenta de Google, con la finalidad de acceder sin crear ni recordar otra contraseña.</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Acceso con Google</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Planificada</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 21-09-2026 (épica E1). Solo Google; el acceso con Apple quedó fuera por decisión del Product Owner. 21-09-2026: en espera del ID de cliente de Google; el botón ya está en las pantallas, desactivado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-17</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario o profesional, necesito elegir mi rol al registrarme, confirmar mi contraseña y decidir si mantener mi sesión iniciada, con la finalidad de acceder a las funciones que me corresponden de forma cómoda y segura.</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Registro con rol y sesión recordada</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 21-09-2026 (épica E1) junto con la nueva identidad visual de las pantallas de acceso (logo, paleta azul y naranja). El registro no incluye la casilla de términos y condiciones. 21-09-2026: implementada y probada (CP-008 a CP-010); falta completar la DoD (revisión de código y PR).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-18</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario, necesito indicar mi objetivo principal y mi estilo de vida (comidas al día y horas de sueño), con la finalidad de recibir una orientación acorde a lo que busco lograr.</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Objetivos y estilo de vida</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 21-09-2026 (épica E1) junto con el asistente de perfil de 4 pasos y el resumen con "Editar" (rediseño de FS-HU-02). 21-09-2026: implementada y probada (CP-018); falta completar la DoD (revisión de código y PR).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-19</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario, necesito registrar mis condiciones médicas, medicamentos y alergias de forma confidencial, con la finalidad de recibir recomendaciones más seguras y adecuadas a mi situación.</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Información de salud</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 21-09-2026 (épica E1). Dato sensible: solo opciones de catálogo, sin texto libre, y solo su dueño lo consulta (DAS, QS7). 21-09-2026: implementada y probada (CP-014 a CP-017); falta completar la DoD (revisión de código y PR).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FS-HU-20 Portada publica: documentacion (DAS v1.11, DoD v1.6, CP-020 a CP-023) y correccion del aviso de cierre de sesion
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I23"/>
+  <dimension ref="B1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" style="5" min="1" max="1"/>
@@ -1239,6 +1239,44 @@
       <c r="I23" s="9" t="inlineStr">
         <is>
           <t>Agregada el 21-09-2026 (épica E1). Dato sensible: solo opciones de catálogo, sin texto libre, y solo su dueño lo consulta (DAS, QS7). 21-09-2026: implementada y probada (CP-014 a CP-017); falta completar la DoD (revisión de código y PR).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-20</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Como un visitante, necesito conocer qué ofrece FitSearch antes de crear una cuenta o iniciar sesión, con la finalidad de decidir si registrarme y acceder fácilmente a la plataforma.</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Portada pública</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 23-09-2026 (épica E1). La portada la construyó Nicolás Silva (PR #2, 22-09-2026); el 23-09-2026 el Product Owner definió que es solo para quien no ha iniciado sesión: con la sesión iniciada se va directo al perfil y al cerrar sesión se vuelve a la portada. 23-09-2026: implementada y probada (CP-020 a CP-023); falta completar la DoD (revisión de código).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cierre del Sprint 1: retrospectiva, aceptacion del PO y revision de codigo aprobada (PR #6)
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I24"/>
+  <dimension ref="B1:I39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" style="5" min="1" max="1"/>
@@ -518,6 +518,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -578,7 +579,7 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
@@ -592,7 +593,11 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr"/>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 1: aceptada por el Product Owner el 24-09-2026 (CP-001 a CP-007 aprobados). Excepción a DoD-03 (sin pull request en el Sprint 1) y revisión de código posterior aprobada por Luis Méndez en el PR #6 (24-09-2026).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="9" t="inlineStr">
@@ -612,7 +617,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
@@ -628,7 +633,7 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Se agregó el sexo a los datos básicos (Sprint 1) para estimar el requerimiento calórico con la ecuación de Mifflin-St Jeor.</t>
+          <t>Se agregó el sexo a los datos básicos (Sprint 1) para estimar el requerimiento calórico con la ecuación de Mifflin-St Jeor. Sprint 1: aceptada por el Product Owner el 24-09-2026 (CP-001 a CP-007 aprobados). Excepción a DoD-03 (sin pull request en el Sprint 1) y revisión de código posterior aprobada por Luis Méndez en el PR #6 (24-09-2026).</t>
         </is>
       </c>
     </row>
@@ -1280,6 +1285,21 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3149606299212598" footer="0.3149606299212598"/>
   <pageSetup orientation="landscape" scale="70"/>

</xml_diff>

<commit_message>
FS-HU-16 y FS-HU-02: inicio de sesion con Google y el tipo de cuenta se elige en el asistente de perfil
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I39"/>
+  <dimension ref="B1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" style="5" min="1" max="1"/>
@@ -518,7 +518,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="8" t="inlineStr">
         <is>
@@ -633,7 +632,7 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Se agregó el sexo a los datos básicos (Sprint 1) para estimar el requerimiento calórico con la ecuación de Mifflin-St Jeor. Sprint 1: aceptada por el Product Owner el 24-09-2026 (CP-001 a CP-007 aprobados). Excepción a DoD-03 (sin pull request en el Sprint 1) y revisión de código posterior aprobada por Luis Méndez en el PR #6 (24-09-2026).</t>
+          <t>Se agregó el sexo a los datos básicos (Sprint 1) para estimar el requerimiento calórico con la ecuación de Mifflin-St Jeor. Sprint 1: aceptada por el Product Owner el 24-09-2026 (CP-001 a CP-007 aprobados). Excepción a DoD-03 (sin pull request en el Sprint 1) y revisión de código posterior aprobada por Luis Méndez en el PR #6 (24-09-2026). 24-09-2026: por decisión del Product Owner se agregó al asistente un primer paso para elegir el tipo de cuenta (usuario o profesional), que antes se elegía en el registro; el asistente queda de 5 pasos. Implementado y probado (CP-027 y CP-028); pendiente la aceptación del Product Owner del criterio nuevo.</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1112,7 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="F20" s="9" t="n">
@@ -1129,7 +1128,7 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1). Solo Google; el acceso con Apple quedó fuera por decisión del Product Owner. 21-09-2026: en espera del ID de cliente de Google; el botón ya está en las pantallas, desactivado.</t>
+          <t>Agregada el 21-09-2026 (épica E1). Solo Google; el acceso con Apple quedó fuera por decisión del Product Owner. 24-09-2026: creada la cuenta fitsearchoficial@gmail.com y el ID de cliente OAuth en Google Cloud; implementada con el botón oficial de Google Identity Services y la verificación del token en el backend (POST /api/auth/google). La aplicación queda en modo de prueba en Google Cloud, con los correos del equipo como usuarios de prueba. Pendiente: ejecutar los casos de prueba manuales CP-024 y CP-025 con la cuenta de Google y completar la DoD (revisión de código y PR). 24-09-2026: entrar con Google ya no define el rol de la cuenta (se creaba con el rol que estuviera marcado en el registro, lo que provocaba equivocaciones); el tipo de cuenta se elige en el perfil.</t>
         </is>
       </c>
     </row>
@@ -1141,12 +1140,12 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Como un usuario o profesional, necesito elegir mi rol al registrarme, confirmar mi contraseña y decidir si mantener mi sesión iniciada, con la finalidad de acceder a las funciones que me corresponden de forma cómoda y segura.</t>
+          <t>Como un usuario o profesional, necesito confirmar mi contraseña al registrarme y decidir si mantener mi sesión iniciada, con la finalidad de acceder de forma cómoda y segura</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Registro con rol y sesión recordada</t>
+          <t>Registro con contraseña confirmada y sesión recordada</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -1167,7 +1166,7 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1) junto con la nueva identidad visual de las pantallas de acceso (logo, paleta azul y naranja). El registro no incluye la casilla de términos y condiciones. 21-09-2026: implementada y probada (CP-008 a CP-010); falta completar la DoD (revisión de código y PR).</t>
+          <t>Agregada el 21-09-2026 (épica E1) junto con la nueva identidad visual de las pantallas de acceso (logo, paleta azul y naranja). El registro no incluye la casilla de términos y condiciones. 21-09-2026: implementada y probada (CP-008 a CP-010); falta completar la DoD (revisión de código y PR). 24-09-2026: se quitó del registro la elección del rol (pasó al asistente de perfil, FS-HU-02); toda cuenta nueva se crea como usuario. CP-008 se rehizo con el flujo nuevo.</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1204,7 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1) junto con el asistente de perfil de 4 pasos y el resumen con "Editar" (rediseño de FS-HU-02). 21-09-2026: implementada y probada (CP-018); falta completar la DoD (revisión de código y PR).</t>
+          <t>Agregada el 21-09-2026 (épica E1) junto con el asistente de perfil de 5 pasos y el resumen con "Editar" (rediseño de FS-HU-02). 21-09-2026: implementada y probada (CP-018); falta completar la DoD (revisión de código y PR).</t>
         </is>
       </c>
     </row>
@@ -1285,21 +1284,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3149606299212598" footer="0.3149606299212598"/>
   <pageSetup orientation="landscape" scale="70"/>

</xml_diff>